<commit_message>
Add quality-of-success, price, player count, comps and competitor results
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJR2Tn3kCW9FarCETGMuGF
</commit_message>
<xml_diff>
--- a/data/competitors.xlsx
+++ b/data/competitors.xlsx
@@ -8,15 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Пояснения" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="A — прямые" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="B — тема + формат" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="C — формат" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ближайшие" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="A — прямые" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="B — тема + формат" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="C — формат" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Пояснения'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'A — прямые'!$A$1:$L$171</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'B — тема + формат'!$A$1:$L$69</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'C — формат'!$A$1:$L$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Пояснения'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Ближайшие'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'A — прямые'!$A$1:$M$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'B — тема + формат'!$A$1:$M$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'C — формат'!$A$1:$M$120</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -483,29 +485,41 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Даты</t>
+          <t>Ближайшие</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Анонсы без конкретной даты («To be announced», «Coming soon») часто заброшены — они в конце каждого листа.</t>
+          <t>15 анонсов, отобранных вручную по описаниям как самые близкие к «собака + охота + кооп».</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Даты</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Анонсы без конкретной даты («To be announced», «Coming soon») часто заброшены — они в конце каждого листа.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Данные</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Steam на 2026-10-04. Без AAA. Вишлисты и подписчики Steam не отдаёт.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -516,7 +530,1054 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="90" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Уровень</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Игра</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Выход</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Издатель</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Собака</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Охота</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Онлайн-кооп</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Стелс</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Хоррор</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Главные теги</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Чем похожа</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blue Ridge Hunting</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Jade Meadows</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Jade &amp;amp; Company</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Horror, Online Co-Op, First-Person, Multiplayer, Survival Horror, Exploration, PvE, Team-Based, Mythology, Co-op Campaign</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Blue Ridge Hunting is a co-op horror game set in the Appalachian Mountains. Solo or with friends, investigate, document, and hunt cryptids based on real sightings, legends, and eerie phenomena from the region. Are you brave enough to uncover the truth?</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2434930/</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>кооп-хоррор: охота на криптидов</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hunting Simulator 3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nacon Studio Ghent</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Nacon</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Hunting, Open World, Simulation, Realistic, First-Person, Singleplayer, Exploration, Nature, Adventure, Action</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>This open-world game lets you experience the thrill of the hunt, with your faithful dog by your side! Choose your equipment from official brands, and explore the wilderness in search of your next game.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2482760/</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>реалистичная охота с собакой, открытый мир</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Meat Safari</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GoblinRunt Games</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GoblinRunt Games</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Online Co-Op, Party Game, Cooking, Driving, Co-op, Physics, Multiplayer, Hunting, Team-Based, Time Management</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Meat Safari is a multiplayer open-world restaurant simulator! Hunt ingredients, cook meat, stack cargo, and race across Meat World solo or in 4-player online co-op. Choose your driver and vehicle, and get out on the safarI!</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/5200400/</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>кооп: охота на ингредиенты + готовка, пати</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hide or Seek: Container Island</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Thia Studio</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Thia Studio; Ozz Games</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Early Access, Online Co-Op, PvE, Adventure, PvP, Action-Adventure, Action, Casual, Family Friendly, Exploration</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Hide or Seek: Container Island is COOP, PVP or solo game where you can hide as a cat or seek as a dog. While hiding, you have to hide through multiple areas in Container Island using magic potions from Dhugs, while evading creatures. While seeking, you have to capture all cats.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4682910/</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>прятки: кошки против собак, кооп/PvP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PAWTENTIAL DISASTER</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yummy Games</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Yummy Games</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Multiplayer, Adventure, Physics, Online Co-Op, Action-Adventure, Co-op, Singleplayer, Exploration, Dogs, Action</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>A chaotic physics co-op game where a pack of dogs must get one very unlucky baby back home and a avoid Pawtential Disaster.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4685480/</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>хаотичный физический кооп за стаю собак</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fearless Crew</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Wise Bu</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Wise Bu</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Exploration, Collectathon, Creature Collector, Hunting, Party Game, Action-Adventure, 3D, First-Person, Horror, Procedural Generation</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Fearless Crew is a  monster-hunter  co-op game where you and up to 3 friends hunt monsters and bring them back to the ship. Each monster is caught in a unique way, with different tools - so be smart about what items you use and when. Even you might get caught off guard by the very tools you use</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4644500/</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>кооп-охота на монстров с выносом добычи на корабль</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Barely Alive</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Sauce Games</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sauce Games</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Action, Party Game, Casual, Online Co-Op, Multiplayer, Survival, Exploration, First-Person, Nature, Snow</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>A co-op survival party game. Hunt your friends or survive until sunrise.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2982710/</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>кооп-выживание, пати: «охоться на друзей»</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dirty Dogs</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2027-03-31</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Zedstar Games</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Zedstar Games</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Social Deduction, Party Game, Multiplayer, Online Co-Op, PvP, Team-Based, Casual, Funny, Cute, Hand-drawn</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>An online party game for 3 to 10 players. Among Us meets Cluedo, in a dog park. Mark your territory, sniff out the strays in disguise, and argue it out at the pack meeting.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/5219680/</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>социальная дедукция за собак (пати)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flow's Island</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Videolud</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Videolud</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Dogs, Multiplayer, Massively Multiplayer, Online Co-Op, Survival, Combat, Open World, Character Customization, PvP, PvE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>You are one of the strays created by a multinational company determined to seize the power that hides on a mysterious island. Collaborate, survive, fight for your place in the pack and discover the magical secret of the tribes living on the Flow's Island.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/1474500/</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>кооп-выживание за бродячих зверей</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>How to Hunt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Rocky Games</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Rocky Games</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Multiplayer, Online Co-Op, Fishing, Co-op, Action, Hunting, Shooter, First-Person, Physics, Adventure</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>A 1-4 player physics based hunting simulator. While drinking and boating you suddenly crash into a small island. To work your way back home you have to learn How to Hunt.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/5235520/</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>физический кооп-симулятор охоты на 1–4 игроков</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fading Day</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ferroclast Games</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ferroclast Games</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Survival Horror, Crafting, RPG, Open World Survival Craft, Adventure, Online Co-Op, Post-apocalyptic, Action, Character Customization, Casual</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Fading Day is an open-world co-op survival horror game. Explore a world changed by an ancient virus, build your shelter, craft, hunt, and survive The Hollowed and mysterious anomalies. Watch your infection, trust your friends, and uncover what lies beneath the ice.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/5303570/</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>кооп-хоррор выживание, есть собака</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Salty Dogs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Crossbridge Game Studios</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Polden Publishing</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Action, Adventure, Co-op, Casual, 2D, Multiplayer, Underwater, Cute, Pixel Graphics, Dogs</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Salty Dogs is a co-op 2D physics-based action game about a squad of badass dogs who arm up and dive into a corrupted ocean. Blast mutated sea life, haul loot back to your submarine, upgrade it between runs, and fight your way down through the dark toward dreadful Cat-o-Cthulhu.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4213930/</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>кооп-отряд вооружённых собак, 2D-экшен</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Quack Hunters</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Coming soon</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Vampire Squid</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Polden Publishing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Multiplayer, Co-op, Funny, Hunting, Online Co-Op, Adventure, Exploration, Action, First-Person, Atmospheric</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>A 1-4 player physics based hunting simulator. A UFO has abducted your grandpa’s beloved goat and irradiated the wildlife in the forest. Gear up, lock and load, and blast your way through the wild to bring your favorite pet home!</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/4252280/</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>физический кооп-симулятор охоты на 1–4 игроков с юмором и хоррором</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ultimate Hunting®</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Wildlands Interactive</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Ultimate Games S.A.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Hunting, Simulation, Nature, Open World, Dogs, Adventure, First-Person, Exploration, Relaxing, Singleplayer</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Where each virtual action captures the true essence of hunting: REAL, BRUTAL, UNFORGETTABLE. Embark on a hunting expedition, returning with valuable trophies and memorable experiences. Customize your gear and adapt your hunting techniques to explore vast, realistic environments.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/1376880/</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>реалистичная охота, есть собака</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Man and Dog</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>To be announced</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Tetrao Studio</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Ultimate Games S.A.; PlayWay S.A.; Ultimate Publishing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Adventure, Hunting, Multiplayer, Dogs, Immersive Sim, Nature, Open World, Realistic, 3D, Online Co-Op</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Man &amp; Dog is a hunting simulation game situated in Finland. Together with your companion dog, use real Nordic hunting methods to seek grouse bird hiding in the trees, or get into a thrilling chase with a fox or rabbit. Immerse yourself in authentic Finnish wilderness in autumm or winter.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://store.steampowered.com/app/2794480/</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>симулятор охоты с собакой, онлайн-кооп</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -531,6 +1592,7 @@
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="90" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -594,6 +1656,11 @@
           <t>Ссылка</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Чем похожа</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -640,6 +1707,7 @@
           <t>https://store.steampowered.com/app/5213150/</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -686,6 +1754,7 @@
           <t>https://store.steampowered.com/app/3064040/</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -738,6 +1807,11 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/2434930/</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>кооп-хоррор: охота на криптидов</t>
         </is>
       </c>
     </row>
@@ -786,6 +1860,7 @@
           <t>https://store.steampowered.com/app/5155810/</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -840,6 +1915,7 @@
           <t>https://store.steampowered.com/app/2174060/</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -890,6 +1966,11 @@
           <t>https://store.steampowered.com/app/2482760/</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>реалистичная охота с собакой, открытый мир</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -940,6 +2021,7 @@
           <t>https://store.steampowered.com/app/5211690/</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -994,6 +2076,7 @@
           <t>https://store.steampowered.com/app/4927030/</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1040,6 +2123,7 @@
           <t>https://store.steampowered.com/app/4634930/</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1090,6 +2174,11 @@
           <t>https://store.steampowered.com/app/5200400/</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>кооп: охота на ингредиенты + готовка, пати</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1142,6 +2231,11 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/4682910/</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>прятки: кошки против собак, кооп/PvP</t>
         </is>
       </c>
     </row>
@@ -1194,6 +2288,11 @@
           <t>https://store.steampowered.com/app/4685480/</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>хаотичный физический кооп за стаю собак</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1250,6 +2349,11 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/4644500/</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>кооп-охота на монстров с выносом добычи на корабль</t>
         </is>
       </c>
     </row>
@@ -1298,6 +2402,7 @@
           <t>https://store.steampowered.com/app/1728620/</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1344,6 +2449,7 @@
           <t>https://store.steampowered.com/app/5035940/</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1394,6 +2500,7 @@
           <t>https://store.steampowered.com/app/5080060/</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1440,6 +2547,7 @@
           <t>https://store.steampowered.com/app/5068870/</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1490,6 +2598,7 @@
           <t>https://store.steampowered.com/app/5025110/</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1540,6 +2649,7 @@
           <t>https://store.steampowered.com/app/5268480/</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1590,6 +2700,7 @@
           <t>https://store.steampowered.com/app/5254220/</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1636,6 +2747,7 @@
           <t>https://store.steampowered.com/app/4782240/</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1686,6 +2798,7 @@
           <t>https://store.steampowered.com/app/4986260/</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1732,6 +2845,7 @@
           <t>https://store.steampowered.com/app/4998160/</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1782,6 +2896,7 @@
           <t>https://store.steampowered.com/app/3664440/</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1832,6 +2947,7 @@
           <t>https://store.steampowered.com/app/3620610/</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1878,6 +2994,7 @@
           <t>https://store.steampowered.com/app/3064500/</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1926,6 +3043,11 @@
       <c r="L28" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/2982710/</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>кооп-выживание, пати: «охоться на друзей»</t>
         </is>
       </c>
     </row>
@@ -1974,6 +3096,7 @@
           <t>https://store.steampowered.com/app/3266120/</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2024,6 +3147,7 @@
           <t>https://store.steampowered.com/app/3828740/</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2078,6 +3202,7 @@
           <t>https://store.steampowered.com/app/3701830/</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2124,6 +3249,7 @@
           <t>https://store.steampowered.com/app/2209340/</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2174,6 +3300,7 @@
           <t>https://store.steampowered.com/app/3990510/</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2220,6 +3347,7 @@
           <t>https://store.steampowered.com/app/4625300/</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2270,6 +3398,7 @@
           <t>https://store.steampowered.com/app/5085900/</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2318,6 +3447,11 @@
       <c r="L36" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/5219680/</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>социальная дедукция за собак (пати)</t>
         </is>
       </c>
     </row>
@@ -2366,6 +3500,7 @@
           <t>https://store.steampowered.com/app/4796520/</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2416,6 +3551,7 @@
           <t>https://store.steampowered.com/app/2751070/</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2466,6 +3602,7 @@
           <t>https://store.steampowered.com/app/3606840/</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2516,6 +3653,7 @@
           <t>https://store.steampowered.com/app/2397360/</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2562,6 +3700,7 @@
           <t>https://store.steampowered.com/app/5136890/</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2608,6 +3747,7 @@
           <t>https://store.steampowered.com/app/3319450/</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2658,6 +3798,7 @@
           <t>https://store.steampowered.com/app/4713940/</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2712,6 +3853,7 @@
           <t>https://store.steampowered.com/app/4393700/</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2762,6 +3904,7 @@
           <t>https://store.steampowered.com/app/5088770/</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2812,6 +3955,7 @@
           <t>https://store.steampowered.com/app/5043650/</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2858,6 +4002,7 @@
           <t>https://store.steampowered.com/app/1334440/</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2912,6 +4057,7 @@
           <t>https://store.steampowered.com/app/4801280/</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2962,6 +4108,7 @@
           <t>https://store.steampowered.com/app/2564480/</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3012,6 +4159,7 @@
           <t>https://store.steampowered.com/app/1940080/</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3062,6 +4210,7 @@
           <t>https://store.steampowered.com/app/3999950/</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3112,6 +4261,7 @@
           <t>https://store.steampowered.com/app/3851160/</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3158,6 +4308,7 @@
           <t>https://store.steampowered.com/app/1504940/</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3209,6 +4360,7 @@
           <t>https://store.steampowered.com/app/4513470/</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3259,6 +4411,7 @@
           <t>https://store.steampowered.com/app/1400560/</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3313,6 +4466,11 @@
           <t>https://store.steampowered.com/app/1474500/</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>кооп-выживание за бродячих зверей</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3367,6 +4525,7 @@
           <t>https://store.steampowered.com/app/1441560/</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3420,6 +4579,7 @@
           <t>https://store.steampowered.com/app/4353520/</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3470,6 +4630,7 @@
           <t>https://store.steampowered.com/app/4361870/</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3524,6 +4685,7 @@
           <t>https://store.steampowered.com/app/1756230/</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3570,6 +4732,7 @@
           <t>https://store.steampowered.com/app/4447410/</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3616,6 +4779,7 @@
           <t>https://store.steampowered.com/app/4487560/</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3670,6 +4834,7 @@
           <t>https://store.steampowered.com/app/4456030/</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3724,6 +4889,7 @@
           <t>https://store.steampowered.com/app/4502820/</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3774,6 +4940,7 @@
           <t>https://store.steampowered.com/app/4444220/</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3820,6 +4987,7 @@
           <t>https://store.steampowered.com/app/1606970/</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3866,6 +5034,7 @@
           <t>https://store.steampowered.com/app/5104280/</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3920,6 +5089,7 @@
           <t>https://store.steampowered.com/app/5106700/</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3974,6 +5144,7 @@
           <t>https://store.steampowered.com/app/5068220/</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4026,6 +5197,7 @@
           <t>https://store.steampowered.com/app/4948090/</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4076,6 +5248,7 @@
           <t>https://store.steampowered.com/app/777210/</t>
         </is>
       </c>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4131,6 +5304,7 @@
           <t>https://store.steampowered.com/app/5231840/</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4183,6 +5357,11 @@
       <c r="L73" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/5235520/</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>физический кооп-симулятор охоты на 1–4 игроков</t>
         </is>
       </c>
     </row>
@@ -4231,6 +5410,7 @@
           <t>https://store.steampowered.com/app/5241470/</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4283,6 +5463,11 @@
       <c r="L75" t="inlineStr">
         <is>
           <t>https://store.steampowered.com/app/5303570/</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>кооп-хоррор выживание, есть собака</t>
         </is>
       </c>
     </row>
@@ -4335,6 +5520,7 @@
           <t>https://store.steampowered.com/app/5161180/</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4386,6 +5572,7 @@
           <t>https://store.steampowered.com/app/1294480/</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4432,6 +5619,7 @@
           <t>https://store.steampowered.com/app/1289180/</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4478,6 +5666,7 @@
           <t>https://store.steampowered.com/app/1329490/</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4524,6 +5713,7 @@
           <t>https://store.steampowered.com/app/1299520/</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4578,6 +5768,7 @@
           <t>https://store.steampowered.com/app/4872770/</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4624,6 +5815,7 @@
           <t>https://store.steampowered.com/app/4978260/</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4670,6 +5862,7 @@
           <t>https://store.steampowered.com/app/1042620/</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4720,6 +5913,7 @@
           <t>https://store.steampowered.com/app/5004550/</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4770,6 +5964,7 @@
           <t>https://store.steampowered.com/app/4904190/</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4825,6 +6020,7 @@
           <t>https://store.steampowered.com/app/1187270/</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4875,6 +6071,7 @@
           <t>https://store.steampowered.com/app/1137980/</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4927,6 +6124,7 @@
           <t>https://store.steampowered.com/app/1141920/</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4973,6 +6171,7 @@
           <t>https://store.steampowered.com/app/3582500/</t>
         </is>
       </c>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5023,6 +6222,7 @@
           <t>https://store.steampowered.com/app/2707540/</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5069,6 +6269,7 @@
           <t>https://store.steampowered.com/app/2688190/</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5115,6 +6316,7 @@
           <t>https://store.steampowered.com/app/2688270/</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5161,6 +6363,7 @@
           <t>https://store.steampowered.com/app/2762970/</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5211,6 +6414,7 @@
           <t>https://store.steampowered.com/app/3651960/</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5269,6 +6473,7 @@
           <t>https://store.steampowered.com/app/3682950/</t>
         </is>
       </c>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5315,6 +6520,7 @@
           <t>https://store.steampowered.com/app/2526300/</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5365,6 +6571,7 @@
           <t>https://store.steampowered.com/app/2550530/</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5415,6 +6622,7 @@
           <t>https://store.steampowered.com/app/3576380/</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5465,6 +6673,7 @@
           <t>https://store.steampowered.com/app/3642500/</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5511,6 +6720,7 @@
           <t>https://store.steampowered.com/app/3018090/</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5557,6 +6767,7 @@
           <t>https://store.steampowered.com/app/3169450/</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5607,6 +6818,7 @@
           <t>https://store.steampowered.com/app/5353370/</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5653,6 +6865,7 @@
           <t>https://store.steampowered.com/app/3373440/</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5703,6 +6916,7 @@
           <t>https://store.steampowered.com/app/2875260/</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5753,6 +6967,7 @@
           <t>https://store.steampowered.com/app/2934340/</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5803,6 +7018,7 @@
           <t>https://store.steampowered.com/app/3297250/</t>
         </is>
       </c>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5857,6 +7073,7 @@
           <t>https://store.steampowered.com/app/4081760/</t>
         </is>
       </c>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5907,6 +7124,7 @@
           <t>https://store.steampowered.com/app/4123960/</t>
         </is>
       </c>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5957,6 +7175,7 @@
           <t>https://store.steampowered.com/app/1998280/</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6003,6 +7222,7 @@
           <t>https://store.steampowered.com/app/4026290/</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6053,6 +7273,7 @@
           <t>https://store.steampowered.com/app/2099570/</t>
         </is>
       </c>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6099,6 +7320,7 @@
           <t>https://store.steampowered.com/app/2068680/</t>
         </is>
       </c>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6145,6 +7367,7 @@
           <t>https://store.steampowered.com/app/4041340/</t>
         </is>
       </c>
+      <c r="M113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6200,6 +7423,7 @@
           <t>https://store.steampowered.com/app/1904830/</t>
         </is>
       </c>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6254,6 +7478,11 @@
           <t>https://store.steampowered.com/app/4213930/</t>
         </is>
       </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>кооп-отряд вооружённых собак, 2D-экшен</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6308,6 +7537,11 @@
           <t>https://store.steampowered.com/app/4252280/</t>
         </is>
       </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>физический кооп-симулятор охоты на 1–4 игроков с юмором и хоррором</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6362,6 +7596,7 @@
           <t>https://store.steampowered.com/app/4254650/</t>
         </is>
       </c>
+      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6408,6 +7643,7 @@
           <t>https://store.steampowered.com/app/1946600/</t>
         </is>
       </c>
+      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6454,6 +7690,7 @@
           <t>https://store.steampowered.com/app/1965070/</t>
         </is>
       </c>
+      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6500,6 +7737,7 @@
           <t>https://store.steampowered.com/app/1916560/</t>
         </is>
       </c>
+      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6550,6 +7788,7 @@
           <t>https://store.steampowered.com/app/3803670/</t>
         </is>
       </c>
+      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6600,6 +7839,7 @@
           <t>https://store.steampowered.com/app/2499750/</t>
         </is>
       </c>
+      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6646,6 +7886,7 @@
           <t>https://store.steampowered.com/app/3701330/</t>
         </is>
       </c>
+      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6698,6 +7939,7 @@
           <t>https://store.steampowered.com/app/2193510/</t>
         </is>
       </c>
+      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6753,6 +7995,7 @@
           <t>https://store.steampowered.com/app/2196020/</t>
         </is>
       </c>
+      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6803,6 +8046,7 @@
           <t>https://store.steampowered.com/app/2329070/</t>
         </is>
       </c>
+      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6849,6 +8093,7 @@
           <t>https://store.steampowered.com/app/2265370/</t>
         </is>
       </c>
+      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6895,6 +8140,7 @@
           <t>https://store.steampowered.com/app/2293400/</t>
         </is>
       </c>
+      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6949,6 +8195,11 @@
           <t>https://store.steampowered.com/app/1376880/</t>
         </is>
       </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>реалистичная охота, есть собака</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6999,6 +8250,7 @@
           <t>https://store.steampowered.com/app/1483770/</t>
         </is>
       </c>
+      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7049,6 +8301,7 @@
           <t>https://store.steampowered.com/app/4313710/</t>
         </is>
       </c>
+      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7099,6 +8352,7 @@
           <t>https://store.steampowered.com/app/4341910/</t>
         </is>
       </c>
+      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7153,6 +8407,7 @@
           <t>https://store.steampowered.com/app/1699180/</t>
         </is>
       </c>
+      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7200,6 +8455,7 @@
           <t>https://store.steampowered.com/app/4270860/</t>
         </is>
       </c>
+      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7246,6 +8502,7 @@
           <t>https://store.steampowered.com/app/1792460/</t>
         </is>
       </c>
+      <c r="M135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7300,6 +8557,7 @@
           <t>https://store.steampowered.com/app/4455810/</t>
         </is>
       </c>
+      <c r="M136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7346,6 +8604,7 @@
           <t>https://store.steampowered.com/app/1545020/</t>
         </is>
       </c>
+      <c r="M137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7397,6 +8656,7 @@
           <t>https://store.steampowered.com/app/1550520/</t>
         </is>
       </c>
+      <c r="M138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7451,6 +8711,7 @@
           <t>https://store.steampowered.com/app/1563250/</t>
         </is>
       </c>
+      <c r="M139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7501,6 +8762,7 @@
           <t>https://store.steampowered.com/app/5026050/</t>
         </is>
       </c>
+      <c r="M140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7547,6 +8809,7 @@
           <t>https://store.steampowered.com/app/5082010/</t>
         </is>
       </c>
+      <c r="M141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7593,6 +8856,7 @@
           <t>https://store.steampowered.com/app/3129180/</t>
         </is>
       </c>
+      <c r="M142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7643,6 +8907,7 @@
           <t>https://store.steampowered.com/app/5219000/</t>
         </is>
       </c>
+      <c r="M143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7695,6 +8960,7 @@
           <t>https://store.steampowered.com/app/5168140/</t>
         </is>
       </c>
+      <c r="M144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7745,6 +9011,7 @@
           <t>https://store.steampowered.com/app/1257610/</t>
         </is>
       </c>
+      <c r="M145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7795,6 +9062,7 @@
           <t>https://store.steampowered.com/app/4909050/</t>
         </is>
       </c>
+      <c r="M146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7849,6 +9117,11 @@
           <t>https://store.steampowered.com/app/2794480/</t>
         </is>
       </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>симулятор охоты с собакой, онлайн-кооп</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7899,6 +9172,7 @@
           <t>https://store.steampowered.com/app/2813510/</t>
         </is>
       </c>
+      <c r="M148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7949,6 +9223,7 @@
           <t>https://store.steampowered.com/app/2744100/</t>
         </is>
       </c>
+      <c r="M149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8000,6 +9275,7 @@
           <t>https://store.steampowered.com/app/2773660/</t>
         </is>
       </c>
+      <c r="M150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8046,6 +9322,7 @@
           <t>https://store.steampowered.com/app/3577240/</t>
         </is>
       </c>
+      <c r="M151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -8092,6 +9369,7 @@
           <t>https://store.steampowered.com/app/3629640/</t>
         </is>
       </c>
+      <c r="M152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8138,6 +9416,7 @@
           <t>https://store.steampowered.com/app/3193580/</t>
         </is>
       </c>
+      <c r="M153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8188,6 +9467,7 @@
           <t>https://store.steampowered.com/app/3031450/</t>
         </is>
       </c>
+      <c r="M154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8234,6 +9514,7 @@
           <t>https://store.steampowered.com/app/2990920/</t>
         </is>
       </c>
+      <c r="M155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8280,6 +9561,7 @@
           <t>https://store.steampowered.com/app/3268910/</t>
         </is>
       </c>
+      <c r="M156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -8326,6 +9608,7 @@
           <t>https://store.steampowered.com/app/3111960/</t>
         </is>
       </c>
+      <c r="M157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -8376,6 +9659,7 @@
           <t>https://store.steampowered.com/app/3148930/</t>
         </is>
       </c>
+      <c r="M158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -8426,6 +9710,7 @@
           <t>https://store.steampowered.com/app/2822720/</t>
         </is>
       </c>
+      <c r="M159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8480,6 +9765,7 @@
           <t>https://store.steampowered.com/app/2861080/</t>
         </is>
       </c>
+      <c r="M160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8526,6 +9812,7 @@
           <t>https://store.steampowered.com/app/2866470/</t>
         </is>
       </c>
+      <c r="M161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8572,6 +9859,7 @@
           <t>https://store.steampowered.com/app/3288340/</t>
         </is>
       </c>
+      <c r="M162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8622,6 +9910,7 @@
           <t>https://store.steampowered.com/app/2957900/</t>
         </is>
       </c>
+      <c r="M163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8672,6 +9961,7 @@
           <t>https://store.steampowered.com/app/1994650/</t>
         </is>
       </c>
+      <c r="M164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8723,6 +10013,7 @@
           <t>https://store.steampowered.com/app/2175180/</t>
         </is>
       </c>
+      <c r="M165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8773,6 +10064,7 @@
           <t>https://store.steampowered.com/app/2084190/</t>
         </is>
       </c>
+      <c r="M166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8819,6 +10111,7 @@
           <t>https://store.steampowered.com/app/4262850/</t>
         </is>
       </c>
+      <c r="M167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8865,6 +10158,7 @@
           <t>https://store.steampowered.com/app/1940360/</t>
         </is>
       </c>
+      <c r="M168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8915,6 +10209,7 @@
           <t>https://store.steampowered.com/app/1929980/</t>
         </is>
       </c>
+      <c r="M169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8965,6 +10260,7 @@
           <t>https://store.steampowered.com/app/3847920/</t>
         </is>
       </c>
+      <c r="M170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -9012,20 +10308,21 @@
           <t>https://store.steampowered.com/app/3976520/</t>
         </is>
       </c>
+      <c r="M171" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L171"/>
+  <autoFilter ref="A1:M171"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9040,6 +10337,7 @@
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="90" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9103,6 +10401,11 @@
           <t>Ссылка</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Чем похожа</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9149,6 +10452,7 @@
           <t>https://store.steampowered.com/app/2254990/</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9199,6 +10503,7 @@
           <t>https://store.steampowered.com/app/5259850/</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9245,6 +10550,7 @@
           <t>https://store.steampowered.com/app/4147720/</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9299,6 +10605,7 @@
           <t>https://store.steampowered.com/app/4132210/</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9345,6 +10652,7 @@
           <t>https://store.steampowered.com/app/4981810/</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9391,6 +10699,7 @@
           <t>https://store.steampowered.com/app/5290350/</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9441,6 +10750,7 @@
           <t>https://store.steampowered.com/app/4132460/</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9491,6 +10801,7 @@
           <t>https://store.steampowered.com/app/2507690/</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9541,6 +10852,7 @@
           <t>https://store.steampowered.com/app/3672980/</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9587,6 +10899,7 @@
           <t>https://store.steampowered.com/app/4033720/</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9633,6 +10946,7 @@
           <t>https://store.steampowered.com/app/4294330/</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9679,6 +10993,7 @@
           <t>https://store.steampowered.com/app/4335960/</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9729,6 +11044,7 @@
           <t>https://store.steampowered.com/app/4480150/</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9781,6 +11097,7 @@
           <t>https://store.steampowered.com/app/4519930/</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9831,6 +11148,7 @@
           <t>https://store.steampowered.com/app/4883760/</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9882,6 +11200,7 @@
           <t>https://store.steampowered.com/app/5011760/</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9936,6 +11255,7 @@
           <t>https://store.steampowered.com/app/5013410/</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9986,6 +11306,7 @@
           <t>https://store.steampowered.com/app/3980790/</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10032,6 +11353,7 @@
           <t>https://store.steampowered.com/app/4925790/</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10078,6 +11400,7 @@
           <t>https://store.steampowered.com/app/1043460/</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10124,6 +11447,7 @@
           <t>https://store.steampowered.com/app/3847390/</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10174,6 +11498,7 @@
           <t>https://store.steampowered.com/app/4887280/</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10220,6 +11545,7 @@
           <t>https://store.steampowered.com/app/2319410/</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10266,6 +11592,7 @@
           <t>https://store.steampowered.com/app/1663330/</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10316,6 +11643,7 @@
           <t>https://store.steampowered.com/app/1805740/</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10362,6 +11690,7 @@
           <t>https://store.steampowered.com/app/1805820/</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10412,6 +11741,7 @@
           <t>https://store.steampowered.com/app/2056510/</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10462,6 +11792,7 @@
           <t>https://store.steampowered.com/app/2268260/</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10512,6 +11843,7 @@
           <t>https://store.steampowered.com/app/2859470/</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10562,6 +11894,7 @@
           <t>https://store.steampowered.com/app/2930840/</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10616,6 +11949,7 @@
           <t>https://store.steampowered.com/app/2996390/</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10670,6 +12004,7 @@
           <t>https://store.steampowered.com/app/3050090/</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10716,6 +12051,7 @@
           <t>https://store.steampowered.com/app/3092850/</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10766,6 +12102,7 @@
           <t>https://store.steampowered.com/app/3166230/</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -10816,6 +12153,7 @@
           <t>https://store.steampowered.com/app/3472960/</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10866,6 +12204,7 @@
           <t>https://store.steampowered.com/app/3547430/</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10912,6 +12251,7 @@
           <t>https://store.steampowered.com/app/3573420/</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10959,6 +12299,7 @@
           <t>https://store.steampowered.com/app/3701310/</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11005,6 +12346,7 @@
           <t>https://store.steampowered.com/app/3789870/</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -11051,6 +12393,7 @@
           <t>https://store.steampowered.com/app/4139890/</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -11101,6 +12444,7 @@
           <t>https://store.steampowered.com/app/4233980/</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -11151,6 +12495,7 @@
           <t>https://store.steampowered.com/app/4269150/</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -11197,6 +12542,7 @@
           <t>https://store.steampowered.com/app/4314290/</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -11247,6 +12593,7 @@
           <t>https://store.steampowered.com/app/4541830/</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -11297,6 +12644,7 @@
           <t>https://store.steampowered.com/app/4607560/</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -11347,6 +12695,7 @@
           <t>https://store.steampowered.com/app/4655080/</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11393,6 +12742,7 @@
           <t>https://store.steampowered.com/app/4910090/</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11443,6 +12793,7 @@
           <t>https://store.steampowered.com/app/4953420/</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11489,6 +12840,7 @@
           <t>https://store.steampowered.com/app/4969400/</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11535,6 +12887,7 @@
           <t>https://store.steampowered.com/app/5163510/</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -11581,6 +12934,7 @@
           <t>https://store.steampowered.com/app/5257900/</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -11632,6 +12986,7 @@
           <t>https://store.steampowered.com/app/908200/</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -11682,6 +13037,7 @@
           <t>https://store.steampowered.com/app/1572000/</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -11728,6 +13084,7 @@
           <t>https://store.steampowered.com/app/2203830/</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -11774,6 +13131,7 @@
           <t>https://store.steampowered.com/app/2590560/</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -11820,6 +13178,7 @@
           <t>https://store.steampowered.com/app/3132610/</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -11870,6 +13229,7 @@
           <t>https://store.steampowered.com/app/3257620/</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -11921,6 +13281,7 @@
           <t>https://store.steampowered.com/app/3473200/</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -11971,6 +13332,7 @@
           <t>https://store.steampowered.com/app/3530640/</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12018,6 +13380,7 @@
           <t>https://store.steampowered.com/app/3640570/</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12072,6 +13435,7 @@
           <t>https://store.steampowered.com/app/3661410/</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12122,6 +13486,7 @@
           <t>https://store.steampowered.com/app/3836380/</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12168,6 +13533,7 @@
           <t>https://store.steampowered.com/app/4011880/</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12218,6 +13584,7 @@
           <t>https://store.steampowered.com/app/4213030/</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -12268,6 +13635,7 @@
           <t>https://store.steampowered.com/app/4661450/</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -12318,6 +13686,7 @@
           <t>https://store.steampowered.com/app/4715980/</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -12364,6 +13733,7 @@
           <t>https://store.steampowered.com/app/4790660/</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -12410,20 +13780,21 @@
           <t>https://store.steampowered.com/app/5251190/</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L69"/>
+  <autoFilter ref="A1:M69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -12438,6 +13809,7 @@
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="90" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12501,6 +13873,11 @@
           <t>Ссылка</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Чем похожа</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -12555,6 +13932,7 @@
           <t>https://store.steampowered.com/app/4101750/</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12609,6 +13987,7 @@
           <t>https://store.steampowered.com/app/2606850/</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12659,6 +14038,7 @@
           <t>https://store.steampowered.com/app/5050950/</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12713,6 +14093,7 @@
           <t>https://store.steampowered.com/app/4936650/</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12767,6 +14148,7 @@
           <t>https://store.steampowered.com/app/5270220/</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12821,6 +14203,7 @@
           <t>https://store.steampowered.com/app/5317740/</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12875,6 +14258,7 @@
           <t>https://store.steampowered.com/app/4736090/</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12929,6 +14313,7 @@
           <t>https://store.steampowered.com/app/5059340/</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12979,6 +14364,7 @@
           <t>https://store.steampowered.com/app/5167460/</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -13029,6 +14415,7 @@
           <t>https://store.steampowered.com/app/910550/</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13083,6 +14470,7 @@
           <t>https://store.steampowered.com/app/4698160/</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13133,6 +14521,7 @@
           <t>https://store.steampowered.com/app/5352690/</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13187,6 +14576,7 @@
           <t>https://store.steampowered.com/app/5239830/</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13241,6 +14631,7 @@
           <t>https://store.steampowered.com/app/2723370/</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13291,6 +14682,7 @@
           <t>https://store.steampowered.com/app/4964620/</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13345,6 +14737,7 @@
           <t>https://store.steampowered.com/app/4643890/</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13399,6 +14792,7 @@
           <t>https://store.steampowered.com/app/3367710/</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13453,6 +14847,7 @@
           <t>https://store.steampowered.com/app/3809820/</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13507,6 +14902,7 @@
           <t>https://store.steampowered.com/app/4295690/</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13561,6 +14957,7 @@
           <t>https://store.steampowered.com/app/4433420/</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13615,6 +15012,7 @@
           <t>https://store.steampowered.com/app/4443820/</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13669,6 +15067,7 @@
           <t>https://store.steampowered.com/app/4703930/</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13723,6 +15122,7 @@
           <t>https://store.steampowered.com/app/5029430/</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13773,6 +15173,7 @@
           <t>https://store.steampowered.com/app/5223650/</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13827,6 +15228,7 @@
           <t>https://store.steampowered.com/app/3082910/</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13881,6 +15283,7 @@
           <t>https://store.steampowered.com/app/3382460/</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13931,6 +15334,7 @@
           <t>https://store.steampowered.com/app/4115520/</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13985,6 +15389,7 @@
           <t>https://store.steampowered.com/app/4228630/</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14035,6 +15440,7 @@
           <t>https://store.steampowered.com/app/4258290/</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14090,6 +15496,7 @@
           <t>https://store.steampowered.com/app/4824910/</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14140,6 +15547,7 @@
           <t>https://store.steampowered.com/app/5016320/</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14194,6 +15602,7 @@
           <t>https://store.steampowered.com/app/5216270/</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14248,6 +15657,7 @@
           <t>https://store.steampowered.com/app/5093060/</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14302,6 +15712,7 @@
           <t>https://store.steampowered.com/app/3058480/</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14356,6 +15767,7 @@
           <t>https://store.steampowered.com/app/3437600/</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14410,6 +15822,7 @@
           <t>https://store.steampowered.com/app/3513120/</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14460,6 +15873,7 @@
           <t>https://store.steampowered.com/app/4908090/</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14517,6 +15931,7 @@
           <t>https://store.steampowered.com/app/1260740/</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14571,6 +15986,7 @@
           <t>https://store.steampowered.com/app/1550130/</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14625,6 +16041,7 @@
           <t>https://store.steampowered.com/app/1641040/</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14679,6 +16096,7 @@
           <t>https://store.steampowered.com/app/1796280/</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14729,6 +16147,7 @@
           <t>https://store.steampowered.com/app/1956730/</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14779,6 +16198,7 @@
           <t>https://store.steampowered.com/app/1969050/</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14833,6 +16253,7 @@
           <t>https://store.steampowered.com/app/1979920/</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14887,6 +16308,7 @@
           <t>https://store.steampowered.com/app/2002730/</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14938,6 +16360,7 @@
           <t>https://store.steampowered.com/app/2020000/</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -14992,6 +16415,7 @@
           <t>https://store.steampowered.com/app/2121550/</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15046,6 +16470,7 @@
           <t>https://store.steampowered.com/app/2137540/</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15100,6 +16525,7 @@
           <t>https://store.steampowered.com/app/2250740/</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15155,6 +16581,7 @@
           <t>https://store.steampowered.com/app/2539870/</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15209,6 +16636,7 @@
           <t>https://store.steampowered.com/app/2549040/</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15259,6 +16687,7 @@
           <t>https://store.steampowered.com/app/2631080/</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15309,6 +16738,7 @@
           <t>https://store.steampowered.com/app/2823240/</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15363,6 +16793,7 @@
           <t>https://store.steampowered.com/app/2870080/</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15419,6 +16850,7 @@
           <t>https://store.steampowered.com/app/2948690/</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -15469,6 +16901,7 @@
           <t>https://store.steampowered.com/app/3203180/</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -15523,6 +16956,7 @@
           <t>https://store.steampowered.com/app/3297290/</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -15577,6 +17011,7 @@
           <t>https://store.steampowered.com/app/3450150/</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -15631,6 +17066,7 @@
           <t>https://store.steampowered.com/app/3605910/</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -15681,6 +17117,7 @@
           <t>https://store.steampowered.com/app/3720040/</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -15731,6 +17168,7 @@
           <t>https://store.steampowered.com/app/3724810/</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -15785,6 +17223,7 @@
           <t>https://store.steampowered.com/app/3783800/</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -15835,6 +17274,7 @@
           <t>https://store.steampowered.com/app/3799570/</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -15889,6 +17329,7 @@
           <t>https://store.steampowered.com/app/3919430/</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -15943,6 +17384,7 @@
           <t>https://store.steampowered.com/app/4062150/</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -15997,6 +17439,7 @@
           <t>https://store.steampowered.com/app/4082940/</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -16047,6 +17490,7 @@
           <t>https://store.steampowered.com/app/4313930/</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -16097,6 +17541,7 @@
           <t>https://store.steampowered.com/app/4341570/</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -16151,6 +17596,7 @@
           <t>https://store.steampowered.com/app/4502890/</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -16201,6 +17647,7 @@
           <t>https://store.steampowered.com/app/4715160/</t>
         </is>
       </c>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -16255,6 +17702,7 @@
           <t>https://store.steampowered.com/app/4891990/</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -16309,6 +17757,7 @@
           <t>https://store.steampowered.com/app/4926050/</t>
         </is>
       </c>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -16359,6 +17808,7 @@
           <t>https://store.steampowered.com/app/4955330/</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -16409,6 +17859,7 @@
           <t>https://store.steampowered.com/app/4977560/</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -16459,6 +17910,7 @@
           <t>https://store.steampowered.com/app/4984780/</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -16509,6 +17961,7 @@
           <t>https://store.steampowered.com/app/4999760/</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -16563,6 +18016,7 @@
           <t>https://store.steampowered.com/app/5000870/</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -16617,6 +18071,7 @@
           <t>https://store.steampowered.com/app/5074510/</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -16671,6 +18126,7 @@
           <t>https://store.steampowered.com/app/5077140/</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -16721,6 +18177,7 @@
           <t>https://store.steampowered.com/app/5088820/</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -16775,6 +18232,7 @@
           <t>https://store.steampowered.com/app/5091280/</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -16825,6 +18283,7 @@
           <t>https://store.steampowered.com/app/5098600/</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -16875,6 +18334,7 @@
           <t>https://store.steampowered.com/app/5106580/</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -16930,6 +18390,7 @@
           <t>https://store.steampowered.com/app/5113760/</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -16984,6 +18445,7 @@
           <t>https://store.steampowered.com/app/5114740/</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17034,6 +18496,7 @@
           <t>https://store.steampowered.com/app/5122120/</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -17088,6 +18551,7 @@
           <t>https://store.steampowered.com/app/5131420/</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -17138,6 +18602,7 @@
           <t>https://store.steampowered.com/app/5183520/</t>
         </is>
       </c>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -17192,6 +18657,7 @@
           <t>https://store.steampowered.com/app/5210970/</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -17242,6 +18708,7 @@
           <t>https://store.steampowered.com/app/5270510/</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -17296,6 +18763,7 @@
           <t>https://store.steampowered.com/app/5282100/</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -17346,6 +18814,7 @@
           <t>https://store.steampowered.com/app/5298910/</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -17396,6 +18865,7 @@
           <t>https://store.steampowered.com/app/1514970/</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -17450,6 +18920,7 @@
           <t>https://store.steampowered.com/app/1644910/</t>
         </is>
       </c>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -17504,6 +18975,7 @@
           <t>https://store.steampowered.com/app/1789110/</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -17558,6 +19030,7 @@
           <t>https://store.steampowered.com/app/2372930/</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -17608,6 +19081,7 @@
           <t>https://store.steampowered.com/app/2427530/</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -17662,6 +19136,7 @@
           <t>https://store.steampowered.com/app/2453430/</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -17716,6 +19191,7 @@
           <t>https://store.steampowered.com/app/2472810/</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -17770,6 +19246,7 @@
           <t>https://store.steampowered.com/app/2572540/</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -17824,6 +19301,7 @@
           <t>https://store.steampowered.com/app/2696960/</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -17874,6 +19352,7 @@
           <t>https://store.steampowered.com/app/2994490/</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -17924,6 +19403,7 @@
           <t>https://store.steampowered.com/app/3034290/</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -17978,6 +19458,7 @@
           <t>https://store.steampowered.com/app/3221070/</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -18028,6 +19509,7 @@
           <t>https://store.steampowered.com/app/3321300/</t>
         </is>
       </c>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -18083,6 +19565,7 @@
           <t>https://store.steampowered.com/app/3688770/</t>
         </is>
       </c>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -18137,6 +19620,7 @@
           <t>https://store.steampowered.com/app/3710560/</t>
         </is>
       </c>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -18191,6 +19675,7 @@
           <t>https://store.steampowered.com/app/3736480/</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -18241,6 +19726,7 @@
           <t>https://store.steampowered.com/app/3803250/</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -18295,6 +19781,7 @@
           <t>https://store.steampowered.com/app/3885940/</t>
         </is>
       </c>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -18345,6 +19832,7 @@
           <t>https://store.steampowered.com/app/3928050/</t>
         </is>
       </c>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -18399,6 +19887,7 @@
           <t>https://store.steampowered.com/app/3996870/</t>
         </is>
       </c>
+      <c r="M113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -18453,6 +19942,7 @@
           <t>https://store.steampowered.com/app/4043580/</t>
         </is>
       </c>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -18507,6 +19997,7 @@
           <t>https://store.steampowered.com/app/4237670/</t>
         </is>
       </c>
+      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -18557,6 +20048,7 @@
           <t>https://store.steampowered.com/app/4511350/</t>
         </is>
       </c>
+      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -18611,6 +20103,7 @@
           <t>https://store.steampowered.com/app/4536700/</t>
         </is>
       </c>
+      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -18665,6 +20158,7 @@
           <t>https://store.steampowered.com/app/4622680/</t>
         </is>
       </c>
+      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -18719,6 +20213,7 @@
           <t>https://store.steampowered.com/app/4653090/</t>
         </is>
       </c>
+      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -18769,9 +20264,10 @@
           <t>https://store.steampowered.com/app/4686110/</t>
         </is>
       </c>
+      <c r="M120" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L120"/>
+  <autoFilter ref="A1:M120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>